<commit_message>
Busca do convite por apelido ou primeiro nome, coluna apelidos e escolha entre convites pelo número de pessoas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JMQbuo913VRtQf26pprQfK
</commit_message>
<xml_diff>
--- a/backend/apps-script/planilha-modelo.xlsx
+++ b/backend/apps-script/planilha-modelo.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -433,6 +433,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,6 +467,11 @@
           <t>crianca</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>apelidos</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -493,7 +499,11 @@
           <t>Maria Exemplo</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Souza</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -521,7 +531,6 @@
           <t>João Exemplo</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -581,7 +590,6 @@
           <t>Ana Teste</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>